<commit_message>
se me olvidaron las imagenes xd
</commit_message>
<xml_diff>
--- a/Taller_Dualidad_Solver_Completo1.xlsx
+++ b/Taller_Dualidad_Solver_Completo1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f66bf0d0917e3adb/Documentos/GitHub/ExcelSolverPL/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="971" documentId="8_{BA39E689-899D-490F-8B8B-B9FE1E44DD6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0C8B954D-59FA-46B5-B5FD-81A0D7AF5D32}"/>
+  <xr:revisionPtr revIDLastSave="978" documentId="8_{BA39E689-899D-490F-8B8B-B9FE1E44DD6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{851CD5BB-925F-43FA-94A8-BC59FFB796CC}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="10455" windowHeight="11625" firstSheet="8" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" firstSheet="9" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="E1 - Primal" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
     <sheet name="E3 - Dual" sheetId="6" r:id="rId10"/>
     <sheet name="E4 - Primal" sheetId="7" r:id="rId11"/>
     <sheet name="Informe de respuestas 1" sheetId="17" r:id="rId12"/>
-    <sheet name="Answer Report 1" sheetId="22" r:id="rId13"/>
+    <sheet name="E4 - Informe Dual" sheetId="22" r:id="rId13"/>
     <sheet name="E4 - Dual" sheetId="8" r:id="rId14"/>
   </sheets>
   <definedNames>
@@ -252,7 +252,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="474" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="474" uniqueCount="159">
   <si>
     <t>Variables</t>
   </si>
@@ -725,13 +725,10 @@
     <t>Tiempo de la solución: 0.078 segundos.</t>
   </si>
   <si>
-    <t>Iteraciones:: 2 Subproblemas: 0</t>
-  </si>
-  <si>
-    <t>Tiempo máximo Ilimitado,  Iteraciones: Unlimited, Precisión 0.000001, Usar escala automática</t>
-  </si>
-  <si>
     <t>Máximo de subproblemas Ilimitado, Máximo de soluciones de enteros Ilimitado, Tolerancia de enteros 1%, Asumir no negativo.</t>
+  </si>
+  <si>
+    <t>Tiempo máximo Ilimitado,  Iteraciones Ilimitado, Precisión 0.000001, Usar escala automática</t>
   </si>
 </sst>
 </file>
@@ -897,7 +894,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -924,13 +921,6 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1333,6 +1323,55 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>600075</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>85725</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>38968</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>48290</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Imagen 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B4F1EDCA-77EA-C7BB-EFE5-C2977B921566}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="600075" y="1885950"/>
+          <a:ext cx="6220693" cy="4763165"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
@@ -2427,7 +2466,7 @@
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" s="7"/>
       <c r="B8" t="s">
-        <v>157</v>
+        <v>145</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
@@ -2442,11 +2481,11 @@
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="B11" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="M12" s="21"/>
+      <c r="M12" s="16"/>
     </row>
     <row r="14" spans="1:13" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
@@ -2454,30 +2493,30 @@
       </c>
     </row>
     <row r="15" spans="1:13" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="17" t="s">
+      <c r="B15" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="C15" s="17" t="s">
+      <c r="C15" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="D15" s="17" t="s">
+      <c r="D15" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="E15" s="17" t="s">
+      <c r="E15" s="9" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="16" spans="1:13" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="16" t="s">
+      <c r="B16" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="C16" s="16" t="s">
+      <c r="C16" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="D16" s="19">
+      <c r="D16" s="8">
         <v>-31.25</v>
       </c>
-      <c r="E16" s="19">
+      <c r="E16" s="8">
         <v>-31.25</v>
       </c>
     </row>
@@ -2487,87 +2526,87 @@
       </c>
     </row>
     <row r="20" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="17" t="s">
+      <c r="B20" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="C20" s="17" t="s">
+      <c r="C20" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="D20" s="17" t="s">
+      <c r="D20" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="E20" s="17" t="s">
+      <c r="E20" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="F20" s="17" t="s">
+      <c r="F20" s="9" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B21" s="18" t="s">
+      <c r="B21" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="C21" s="18" t="s">
+      <c r="C21" s="10" t="s">
         <v>106</v>
       </c>
-      <c r="D21" s="20">
+      <c r="D21" s="10">
         <v>0.125</v>
       </c>
-      <c r="E21" s="20">
+      <c r="E21" s="10">
         <v>0.125</v>
       </c>
-      <c r="F21" s="18" t="s">
+      <c r="F21" s="10" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B22" s="18" t="s">
+      <c r="B22" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="C22" s="18" t="s">
+      <c r="C22" s="10" t="s">
         <v>107</v>
       </c>
-      <c r="D22" s="20">
-        <v>0</v>
-      </c>
-      <c r="E22" s="20">
-        <v>0</v>
-      </c>
-      <c r="F22" s="18" t="s">
+      <c r="D22" s="10">
+        <v>0</v>
+      </c>
+      <c r="E22" s="10">
+        <v>0</v>
+      </c>
+      <c r="F22" s="10" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B23" s="18" t="s">
+      <c r="B23" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="C23" s="18" t="s">
+      <c r="C23" s="10" t="s">
         <v>108</v>
       </c>
-      <c r="D23" s="20">
-        <v>0</v>
-      </c>
-      <c r="E23" s="20">
-        <v>0</v>
-      </c>
-      <c r="F23" s="18" t="s">
+      <c r="D23" s="10">
+        <v>0</v>
+      </c>
+      <c r="E23" s="10">
+        <v>0</v>
+      </c>
+      <c r="F23" s="10" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="16" t="s">
+      <c r="B24" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="C24" s="16" t="s">
+      <c r="C24" s="8" t="s">
         <v>149</v>
       </c>
-      <c r="D24" s="19">
+      <c r="D24" s="8">
         <v>6.625</v>
       </c>
-      <c r="E24" s="19">
+      <c r="E24" s="8">
         <v>6.625</v>
       </c>
-      <c r="F24" s="16" t="s">
+      <c r="F24" s="8" t="s">
         <v>50</v>
       </c>
     </row>
@@ -2577,82 +2616,82 @@
       </c>
     </row>
     <row r="28" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="17" t="s">
+      <c r="B28" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="C28" s="17" t="s">
+      <c r="C28" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="D28" s="17" t="s">
+      <c r="D28" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="E28" s="17" t="s">
+      <c r="E28" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="F28" s="17" t="s">
+      <c r="F28" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="G28" s="17" t="s">
+      <c r="G28" s="9" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B29" s="18" t="s">
+      <c r="B29" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="C29" s="18" t="s">
+      <c r="C29" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="D29" s="20">
+      <c r="D29" s="10">
         <v>-6.5</v>
       </c>
-      <c r="E29" s="18" t="s">
+      <c r="E29" s="10" t="s">
         <v>150</v>
       </c>
-      <c r="F29" s="18" t="s">
+      <c r="F29" s="10" t="s">
         <v>139</v>
       </c>
-      <c r="G29" s="18">
+      <c r="G29" s="10">
         <v>11.5</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B30" s="18" t="s">
+      <c r="B30" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="C30" s="18" t="s">
+      <c r="C30" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="D30" s="20">
+      <c r="D30" s="10">
         <v>-6</v>
       </c>
-      <c r="E30" s="18" t="s">
+      <c r="E30" s="10" t="s">
         <v>151</v>
       </c>
-      <c r="F30" s="18" t="s">
+      <c r="F30" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="G30" s="18">
+      <c r="G30" s="10">
         <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="16" t="s">
+      <c r="B31" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="C31" s="16" t="s">
+      <c r="C31" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="D31" s="19">
+      <c r="D31" s="8">
         <v>-7</v>
       </c>
-      <c r="E31" s="16" t="s">
+      <c r="E31" s="8" t="s">
         <v>152</v>
       </c>
-      <c r="F31" s="16" t="s">
+      <c r="F31" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="G31" s="16">
+      <c r="G31" s="8">
         <v>0</v>
       </c>
     </row>
@@ -2861,10 +2900,7 @@
       <c r="A8" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="2">
-        <f>SUMPRODUCT($B$2:$E$2,B7:E7)</f>
-        <v>-31.25</v>
-      </c>
+      <c r="B8" s="2"/>
       <c r="C8" s="3"/>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
@@ -2876,6 +2912,7 @@
   </sheetData>
   <phoneticPr fontId="9" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>